<commit_message>
Expand sample guests to 200 names
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample-guests.xlsx
+++ b/sample-guests.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A201"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,97 +406,1007 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Emma Johnson</v>
+        <v>Caroline Rodriguez</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Liam Smith</v>
+        <v>Emma Ward</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Olivia Williams</v>
+        <v>Zoe James</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Noah Brown</v>
+        <v>Evelyn Nguyen</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ava Davis</v>
+        <v>Caroline Williams</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sophia Wilson</v>
+        <v>Maverick Cooper</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>James Garcia</v>
+        <v>Layla Morgan</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Isabella Martinez</v>
+        <v>Christopher Murphy</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Mason Anderson</v>
+        <v>Jayden Hill</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Mia Taylor</v>
+        <v>Aria Adams</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Ethan Thomas</v>
+        <v>Natalie Castillo</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Charlotte Lee</v>
+        <v>Olivia Walker</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Benjamin Harris</v>
+        <v>Nathan Nelson</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Amelia Clark</v>
+        <v>Harper Bennett</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Lucas Lewis</v>
+        <v>Addison Cox</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Harper Robinson</v>
+        <v>Ellie Lewis</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Alexander Walker</v>
+        <v>Zoe Davis</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Evelyn Hall</v>
+        <v>Evelyn Taylor</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Joseph Hernandez</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Charles Bennett</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Avery Kelly</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Michael Ward</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Sophia Campbell</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Ella Torres</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>James Kelly</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Alexander Wilson</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Mateo Gray</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Genesis Lopez</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>David King</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Matthew Morgan</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Michael Reed</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Ethan Foster</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Zoe Lee</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Julian Johnson</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>James Sanders</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Anna Collins</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Gabriel Scott</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Aiden Harris</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Aiden Davis</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Grace Campbell</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Owen Robinson</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Amelia Bailey</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Levi Jackson</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Harper Diaz</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Kennedy Thomas</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Andrew Brooks</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Abigail Price</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Julian Ramos</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Ezra Kim</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Layla Hughes</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Hazel Baker</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Andrew Diaz</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Elizabeth King</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Sofia Sanders</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>David Johnson</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Kennedy Reed</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Genesis Mendoza</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Sebastian Anderson</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Aria Mitchell</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Jaxon Wilson</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Paisley Ward</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Logan Smith</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Aaliyah Watson</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Addison Gray</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Levi Ruiz</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Kennedy Richardson</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Aiden Long</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Zoe Cook</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Gabriel Thomas</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Joseph Myers</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Ryan Gutierrez</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Christopher Stewart</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Liam Richardson</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Benjamin Ramirez</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Anna Patel</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Claire Cook</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Nathan Flores</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Kennedy Wright</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Claire Young</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Victoria Hernandez</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Ava Bailey</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Jayden Cooper</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Charlotte Patel</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Dylan Rivera</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Jaxon Johnson</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Layla Gomez</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Natalie Davis</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Joshua Robinson</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Andrew Wilson</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Addison Hughes</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Jack Reed</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Natalie Chavez</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Matthew Morris</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Victoria Campbell</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Mia Garcia</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Mia Myers</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Ezra Castillo</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Riley Cruz</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Aria Johnson</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Carter Jimenez</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Lucas Lee</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Paisley Wright</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Lily Carter</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Caroline Foster</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Josiah Nguyen</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Claire Jones</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Aria Morris</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Lucy Ramos</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Sebastian Allen</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Grace Thomas</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Kennedy Collins</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Ava Morris</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Elizabeth Smith</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Levi Parker</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Nora Sanchez</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Eleanor Adams</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Ryan Bennett</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Ella Stewart</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Victoria Price</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Zoe Ruiz</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Ethan Morgan</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Sophia Edwards</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Paisley Perez</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Ella Smith</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Emily Wright</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Abigail Sanchez</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Alexander Alvarez</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>David Rivera</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Audrey Martinez</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Noah Brooks</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Miles Myers</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Hazel Robinson</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Jayden Wright</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>Thomas Allen</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>Eleanor Hill</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Charles Morris</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Joshua Gray</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Jaxon Brown</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>Elijah Jimenez</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>Addison Cook</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>Claire Turner</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>Isabella Cruz</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>Claire Scott</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>Lucas Robinson</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>Jayden Harris</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>Jack Gonzalez</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>Lillian Stewart</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>Logan Wilson</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>Victoria Rivera</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>Addison Harris</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>Aria Ward</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>Audrey Ramirez</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>Carter Davis</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>Isabella Green</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>Benjamin Ward</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>Mateo Jones</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>Aaliyah Diaz</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>Joseph Miller</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>Jacob James</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>Riley Hughes</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>James King</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Christopher Wood</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>Ellie Richardson</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>Audrey Cox</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Maverick Baker</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>Nora Clark</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>David Evans</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>Benjamin Nelson</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>Harper Scott</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>Owen Brooks</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>Zoe Howard</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>John Cox</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>Harper Rodriguez</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>Mateo Brown</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>Addison Davis</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>Audrey Robinson</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>Miles Kim</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>Josiah Clark</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>Benjamin Mendoza</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Zoe Castillo</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Aiden Young</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>Gabriel Allen</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>Grayson Allen</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Amelia Brown</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>Ella Patel</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>Jayden Nguyen</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>Levi Torres</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>Hazel Reed</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>Zoey Torres</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>Wyatt Wilson</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>Ellie Torres</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>Penelope Campbell</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>Savannah Peterson</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Emma Sanders</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Henry Brooks</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Evelyn Harris</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>Mia Watson</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>Ryan Collins</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>Harper Myers</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>Henry Rivera</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A201"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>